<commit_message>
Updated .gitignore to ignore .bak again
</commit_message>
<xml_diff>
--- a/To Add v2/Protection - TVS Diode.xlsx
+++ b/To Add v2/Protection - TVS Diode.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\Danakil_KiCad_DB\To Add v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77DD4282-ED25-4823-B27E-6B9B47CBA9F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0BB0804-36E4-47F0-A112-3031D0EE2ACC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="7725" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="63">
   <si>
     <t>Totals</t>
   </si>
@@ -207,6 +207,24 @@
   </si>
   <si>
     <t>0Dan_Protection:D_TVS_Dual</t>
+  </si>
+  <si>
+    <t>ESD862DBZR</t>
+  </si>
+  <si>
+    <t>Texas Instruments</t>
+  </si>
+  <si>
+    <t>296-ESD862DBZRCT-ND</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/lit/ds/symlink/esd852.pdf?ts=1704443610903</t>
+  </si>
+  <si>
+    <t>2.6pF@1Mhz</t>
+  </si>
+  <si>
+    <t>0Dan_Protection:D_TVS_Dual_2</t>
   </si>
 </sst>
 </file>
@@ -552,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:AB9"/>
+  <dimension ref="B1:AB10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="43.54296875" bestFit="1" customWidth="1"/>
@@ -580,75 +598,75 @@
       </c>
       <c r="C2">
         <f>COUNTA(C7:C9999)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2">
         <f t="shared" ref="D2:T2" si="0">COUNTA(D7:D9999)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F2">
         <f t="shared" ref="F2" si="1">COUNTA(F7:F9999)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2">
         <f t="shared" ref="G2:L2" si="2">COUNTA(G7:G9999)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H2">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I2">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J2">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K2">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L2">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T2">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AA2" t="s">
         <v>1</v>
@@ -665,7 +683,7 @@
       </c>
       <c r="AB3">
         <f>MAX(C2:T2)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="2:28" x14ac:dyDescent="0.35">
@@ -731,7 +749,7 @@
       </c>
       <c r="AB4">
         <f>SUM(Y7:Y9999)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:28" x14ac:dyDescent="0.35">
@@ -1011,6 +1029,88 @@
       </c>
       <c r="T9" t="s">
         <v>35</v>
+      </c>
+      <c r="W9">
+        <f>COUNTBLANK(C9:T9)</f>
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <f>100*COUNTA(C9:T9)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y9">
+        <f>IF(X9=100,1,0)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:28" x14ac:dyDescent="0.35">
+      <c r="C10" t="str">
+        <f>_xlfn.CONCAT(D10," ",I10,"A ",L10," ",T10)</f>
+        <v>Zener 2Ch Bidir 35V 3.1A    </v>
+      </c>
+      <c r="D10" t="str">
+        <f t="shared" ref="D10" si="4">_xlfn.CONCAT(E10," ",F10,"Ch ",G10," ",H10,"V")</f>
+        <v>Zener 2Ch Bidir 35V</v>
+      </c>
+      <c r="E10" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10">
+        <v>35</v>
+      </c>
+      <c r="I10">
+        <v>3.1</v>
+      </c>
+      <c r="J10">
+        <v>175</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M10" t="s">
+        <v>58</v>
+      </c>
+      <c r="N10" t="s">
+        <v>57</v>
+      </c>
+      <c r="O10" t="s">
+        <v>25</v>
+      </c>
+      <c r="P10" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>60</v>
+      </c>
+      <c r="R10" t="s">
+        <v>62</v>
+      </c>
+      <c r="S10" t="s">
+        <v>47</v>
+      </c>
+      <c r="T10" t="s">
+        <v>35</v>
+      </c>
+      <c r="W10">
+        <f>COUNTBLANK(C10:T10)</f>
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <f>100*COUNTA(C10:T10)/$AB$7</f>
+        <v>100</v>
+      </c>
+      <c r="Y10">
+        <f>IF(X10=100,1,0)</f>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1024,6 +1124,7 @@
     <hyperlink ref="K8" r:id="rId2" xr:uid="{41297C62-6D6E-42EF-9ABA-3CFEE4736466}"/>
     <hyperlink ref="Q7" r:id="rId3" xr:uid="{4411BFB1-B34B-49AA-B9D8-ED8BBCDDEEA7}"/>
     <hyperlink ref="Q8" r:id="rId4" xr:uid="{408C4100-39C8-4133-A3B5-D3EE1C6C1ED8}"/>
+    <hyperlink ref="K10" r:id="rId5" xr:uid="{22A9EC77-91D1-47BC-8C90-6C1D4CC7AD85}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>